<commit_message>
Deploying to gh-pages from  @ 9f7a6bfdb3a97b277ca08da6987ba86e5371b789 🚀
</commit_message>
<xml_diff>
--- a/assets/excel/2025_1-1-1.xlsx
+++ b/assets/excel/2025_1-1-1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\github\MT_Site\assets\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D69D8712-84AF-4C13-B957-95BBFBC9D842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA448782-1856-4A6B-B77C-4DD9BAEE1BFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{10A5E901-1E3B-4FD8-A95C-5E70FBB58270}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{10A5E901-1E3B-4FD8-A95C-5E70FBB58270}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -31,6 +31,9 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -337,7 +340,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -428,6 +431,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -435,7 +447,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -511,6 +523,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -5190,6 +5203,9 @@
         <v>-4.5549441069879661E-2</v>
       </c>
     </row>
+    <row r="63" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="C63" s="27"/>
+    </row>
     <row r="64" spans="2:26" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C64" s="9" t="s">
         <v>10</v>

</xml_diff>